<commit_message>
Distingue visuellement les ajouts des retraits dans la grille
La grille de la feuille de lecture encadrait toute cellule portant un ecart
d'une meme bordure rouge. Elle utilise desormais deux regles : bordure VERTE
pour une cellule contenant un ajout "(+...)", bordure ROUGE pour un retrait
"(-...)". La regle du retrait est prioritaire, donc une cellule portant les
deux reste encadree en rouge. La legende de la grille est mise a jour.

Sur la feuille des vols additionnels, les lignes d'ajout prennent un fond vert
clair, en symetrie du fond rose deja applique aux lignes de retrait.

Verifie apres recalcul : 0 erreur sur 3726 formules, regles de bordure ecrites
avec la bonne priorite (retrait en priorite 2, ajout en priorite 3).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sb1vN2YaJtVprJQ5KpgKit
</commit_message>
<xml_diff>
--- a/Programme_vols_mensuel_2027-2028.xlsx
+++ b/Programme_vols_mensuel_2027-2028.xlsx
@@ -315,7 +315,7 @@
     <t xml:space="preserve">Nb de semaines calendaires du mois</t>
   </si>
   <si>
-    <t xml:space="preserve">Lecture : 1re ligne = les rotations qui PARTENT ce jour-la ("2xA320" = deux rotations A320)  |  2e ligne "&lt; 787" = les RETOURS du jour  |  "(+787)" ou "(-787)" encadre en rouge = ajout ou retrait saisi sur la feuille Vols additionnels.</t>
+    <t xml:space="preserve">Lecture : 1re ligne = les rotations qui PARTENT ce jour-la ("2xA320" = deux rotations A320)  |  2e ligne "&lt; 787" = les RETOURS du jour  |  cellule encadree en VERT = vol AJOUTE "(+787)", encadree en ROUGE = vol RETIRE "(-787)", saisis sur la feuille Vols additionnels.</t>
   </si>
   <si>
     <t xml:space="preserve">77W : code du mois precedent</t>
@@ -1767,7 +1767,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="19">
     <dxf>
       <border diagonalUp="false" diagonalDown="false">
         <left style="medium">
@@ -1781,6 +1781,23 @@
         </top>
         <bottom style="medium">
           <color rgb="FFC00000"/>
+        </bottom>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="medium">
+          <color rgb="FF00B050"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF00B050"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF00B050"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF00B050"/>
         </bottom>
         <diagonal/>
       </border>
@@ -2017,6 +2034,13 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <colors>
     <indexedColors>
@@ -2025,7 +2049,7 @@
       <rgbColor rgb="FFC00000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFF2E4D8"/>
+      <rgbColor rgb="FFC6E0B4"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
@@ -2041,12 +2065,12 @@
       <rgbColor rgb="FFFFF2CC"/>
       <rgbColor rgb="FFF2F2F2"/>
       <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFE7E6E6"/>
+      <rgbColor rgb="FFFCE4E4"/>
       <rgbColor rgb="FF0563C1"/>
       <rgbColor rgb="FFD9D2E9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFCE4E4"/>
+      <rgbColor rgb="FFF2E4D8"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF800000"/>
@@ -2054,22 +2078,22 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFD9E2F3"/>
-      <rgbColor rgb="FFC6E0B4"/>
+      <rgbColor rgb="FFE2EFDA"/>
       <rgbColor rgb="FFFFE699"/>
       <rgbColor rgb="FF9DC3E6"/>
       <rgbColor rgb="FFF4B183"/>
       <rgbColor rgb="FFB7DEE8"/>
       <rgbColor rgb="FFFFC7CE"/>
       <rgbColor rgb="FF2E75B6"/>
-      <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FFA9D08E"/>
+      <rgbColor rgb="FF70AD47"/>
       <rgbColor rgb="FFFFD966"/>
-      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFE7E6E6"/>
       <rgbColor rgb="FFED7D31"/>
       <rgbColor rgb="FF595959"/>
       <rgbColor rgb="FFA6A6A6"/>
       <rgbColor rgb="FF1F3864"/>
-      <rgbColor rgb="FF70AD47"/>
+      <rgbColor rgb="FF00B050"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF375623"/>
       <rgbColor rgb="FF833C0C"/>
@@ -6747,80 +6771,83 @@
   </mergeCells>
   <conditionalFormatting sqref="C8:I8 C10:I10 C12:I12 C14:I14 C16:I16 C18:I18">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>ISNUMBER(SEARCH("(",C8))</formula>
+      <formula>ISNUMBER(SEARCH("(-",C8))</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>ISNUMBER(SEARCH("(+",C8))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>AND($C$5="CDGRUN",C8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>AND($C$5="CDGDZA",C8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>AND($C$5="BKKRUN",C8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>AND($C$5="DZARUN",C8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>AND($C$5="MRURUN",C8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>AND($C$5="NOSRUN",C8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>AND($C$5="RUNTNR",C8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>AND($C$5="JNBRUN",C8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>AND($C$5="CPTRUN",C8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>AND($C$5="DIERUN",C8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>AND($C$5="RRGRUN",C8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>AND($C$5="TMMRUN",C8&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25:B36">
-    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>$B25="CDGRUN"</formula>
     </cfRule>
-    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>$B25="CDGDZA"</formula>
     </cfRule>
-    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>$B25="BKKRUN"</formula>
     </cfRule>
-    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>$B25="DZARUN"</formula>
     </cfRule>
-    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>$B25="MRURUN"</formula>
     </cfRule>
-    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>$B25="NOSRUN"</formula>
     </cfRule>
-    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$B25="RUNTNR"</formula>
     </cfRule>
-    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$B25="JNBRUN"</formula>
     </cfRule>
-    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$B25="CPTRUN"</formula>
     </cfRule>
-    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$B25="DIERUN"</formula>
     </cfRule>
-    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$B25="RRGRUN"</formula>
     </cfRule>
-    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="expression" priority="27" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>$B25="TMMRUN"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17475,70 +17502,70 @@
     <mergeCell ref="L475:L477"/>
   </mergeCells>
   <conditionalFormatting sqref="D13:J48 D52:J87 D91:J126 D130:J165 D169:J204 D208:J243 D247:J282 D286:J321 D325:J360 D364:J399 D403:J438 D442:J477">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>LEN(D13)&gt;1</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>D13&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:L11">
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="avril 2027"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B50:L50">
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="mai 2027"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B89:L89">
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="juin 2027"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B128:L128">
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="juillet 2027"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B167:L167">
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="aout 2027"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B206:L206">
-    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="septembre 2027"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B245:L245">
-    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="octobre 2027"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B284:L284">
-    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="novembre 2027"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B323:L323">
-    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="decembre 2027"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B362:L362">
-    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="janvier 2028"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B401:L401">
-    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="fevrier 2028"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B440:L440">
-    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>$C$6="mars 2028"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19183,8 +19210,11 @@
     <mergeCell ref="B2:G4"/>
   </mergeCells>
   <conditionalFormatting sqref="B7:G66">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>$E7&lt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+      <formula>$E7&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">

</xml_diff>